<commit_message>
Site structure: College pages directly under /en, unit sites keep their slug
Mirror lsa.umich.edu under the language root: the College site's pages
(/lsa/...) sit directly below /en (/en/about, /en/prospective-students/...),
department/unit sites keep their slug (/en/english/undergraduate, /en/psych/...,
/en/rc), nav/footer at /en/nav, /en/footer.

- tools/importer/doc-path.mjs: shared source URL -> document path mapping
- import scripts write documents at their final /en path
- build-da-docs.mjs reads only the language root; links, section-nav and
  redirects use doc-path.mjs; redirects cover /lsa/... and /en/lsa/...;
  scheme-less email links get mailto:
- section-nav block: keep off-site entries as absolute links (they were
  reduced to a path and 404'd on this site)
- remove the retired nav-footer importer and localhost URL lists, and the
  import reports for the old document paths

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about.report.xlsx
+++ b/tools/importer/reports/import-about.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="272">
   <si>
     <t>_reportFile</t>
   </si>
@@ -64,7 +64,7 @@
     <t>department-landing</t>
   </si>
   <si>
-    <t>2026-10-07T16:51:52.930Z</t>
+    <t>2026-10-07T16:54:47.551Z</t>
   </si>
   <si>
     <t>Center for Global and Intercultural Study | U-M LSA</t>
@@ -79,7 +79,7 @@
     <t>footer</t>
   </si>
   <si>
-    <t>2026-10-07T16:48:04.163Z</t>
+    <t>2026-10-07T16:56:47.899Z</t>
   </si>
   <si>
     <t>https://lsa.umich.edu/</t>
@@ -151,7 +151,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-10-07T16:47:57.765Z</t>
+    <t>2026-10-07T18:44:48.172Z</t>
   </si>
   <si>
     <t>rc.report.json</t>
@@ -166,7 +166,7 @@
     <t>unit-home</t>
   </si>
   <si>
-    <t>2026-10-07T16:51:39.228Z</t>
+    <t>2026-10-07T16:54:34.133Z</t>
   </si>
   <si>
     <t>Residential College | U-M LSA</t>
@@ -175,13 +175,43 @@
     <t>https://lsa.umich.edu/rc</t>
   </si>
   <si>
+    <t>en/about.report.json</t>
+  </si>
+  <si>
+    <t>["hero","columns","columns","columns","columns","columns","cards"]</t>
+  </si>
+  <si>
+    <t>en/about</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>2026-10-08T13:09:08.323Z</t>
+  </si>
+  <si>
+    <t>About | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/about.html</t>
+  </si>
+  <si>
     <t>en/footer.report.json</t>
   </si>
   <si>
     <t>en/footer</t>
   </si>
   <si>
-    <t>2026-10-07T15:47:50.687Z</t>
+    <t>2026-10-08T13:09:00.952Z</t>
+  </si>
+  <si>
+    <t>en/index.report.json</t>
+  </si>
+  <si>
+    <t>en/index</t>
+  </si>
+  <si>
+    <t>2026-10-08T13:08:47.940Z</t>
   </si>
   <si>
     <t>en/nav.report.json</t>
@@ -190,7 +220,7 @@
     <t>en/nav</t>
   </si>
   <si>
-    <t>2026-10-07T15:47:46.487Z</t>
+    <t>2026-10-08T13:08:55.098Z</t>
   </si>
   <si>
     <t>english/undergraduate.report.json</t>
@@ -202,7 +232,7 @@
     <t>english/undergraduate</t>
   </si>
   <si>
-    <t>2026-10-07T16:51:45.450Z</t>
+    <t>2026-10-07T16:54:40.634Z</t>
   </si>
   <si>
     <t>Undergraduate Students | U-M LSA English Language and Literature</t>
@@ -214,24 +244,12 @@
     <t>lsa/about.report.json</t>
   </si>
   <si>
-    <t>["hero","columns","columns","columns","columns","columns","cards"]</t>
-  </si>
-  <si>
     <t>lsa/about</t>
   </si>
   <si>
-    <t>about</t>
-  </si>
-  <si>
     <t>2026-10-07T16:54:28.368Z</t>
   </si>
   <si>
-    <t>About | U-M LSA U-M College of LSA</t>
-  </si>
-  <si>
-    <t>https://lsa.umich.edu/lsa/about.html</t>
-  </si>
-  <si>
     <t>lsa/prospective-students.report.json</t>
   </si>
   <si>
@@ -259,7 +277,7 @@
     <t>urop/prospective-students</t>
   </si>
   <si>
-    <t>2026-10-07T16:51:48.053Z</t>
+    <t>2026-10-07T16:54:42.605Z</t>
   </si>
   <si>
     <t>Prospective UROP Students | U-M LSA UROP: A Center for Research, Scholarship, and Creative Inquiry</t>
@@ -326,6 +344,84 @@
     <t>https://lsa.umich.edu/lsa/academics/majors-minors.html</t>
   </si>
   <si>
+    <t>lsa/prospective-students/graduate.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate</t>
+  </si>
+  <si>
+    <t>section-interior</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:25.691Z</t>
+  </si>
+  <si>
+    <t>Graduate | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/graduate.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:29.784Z</t>
+  </si>
+  <si>
+    <t>International | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:34.695Z</t>
+  </si>
+  <si>
+    <t>LSA 101: Info for Admitted Students | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:31.755Z</t>
+  </si>
+  <si>
+    <t>Student Stories | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/transfer.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/transfer</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:27.283Z</t>
+  </si>
+  <si>
+    <t>Transfer | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/transfer.html</t>
+  </si>
+  <si>
     <t>lsa/prospective-students/undergraduate.report.json</t>
   </si>
   <si>
@@ -344,19 +440,406 @@
     <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate.html</t>
   </si>
   <si>
+    <t>lsa/prospective-students/visit-campus.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/visit-campus</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:36.357Z</t>
+  </si>
+  <si>
+    <t>Visit Campus | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/visit-campus.html</t>
+  </si>
+  <si>
     <t>psych/prospective-students/undergraduate.report.json</t>
   </si>
   <si>
     <t>psych/prospective-students/undergraduate</t>
   </si>
   <si>
-    <t>2026-10-07T16:51:50.588Z</t>
+    <t>2026-10-07T16:54:44.387Z</t>
   </si>
   <si>
     <t>Undergraduate | U-M LSA Department of Psychology</t>
   </si>
   <si>
     <t>https://lsa.umich.edu/psych/prospective-students/undergraduate.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/applying.report.json</t>
+  </si>
+  <si>
+    <t>["accordion"]</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/applying</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:40.832Z</t>
+  </si>
+  <si>
+    <t>Applying | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/graduate/applying.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/frequently-asked-questions.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/frequently-asked-questions</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:45.514Z</t>
+  </si>
+  <si>
+    <t>Frequently Asked Questions | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/graduate/frequently-asked-questions.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/funding-support.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/graduate/funding-support</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:43.327Z</t>
+  </si>
+  <si>
+    <t>Funding and Support | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/graduate/funding-support.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:48.167Z</t>
+  </si>
+  <si>
+    <t>International Visiting | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/community.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/community</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:06.118Z</t>
+  </si>
+  <si>
+    <t>Community | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/community.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/curriculum.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/curriculum</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:02.247Z</t>
+  </si>
+  <si>
+    <t>Curriculum | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/curriculum.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/events.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/events</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:13.487Z</t>
+  </si>
+  <si>
+    <t>Events | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/events.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/faculty-and-research.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/faculty-and-research</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:04.295Z</t>
+  </si>
+  <si>
+    <t>Faculty and Research | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/faculty-and-research.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/opportunities-beyond-the-classroom.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/opportunities-beyond-the-classroom</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:11.815Z</t>
+  </si>
+  <si>
+    <t>Opportunities Beyond the Classroom | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/opportunities-beyond-the-classroom.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/student-ambassadors.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/lsa101/student-ambassadors</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:32:09.024Z</t>
+  </si>
+  <si>
+    <t>Student Ambassadors | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/lsa101/student-ambassadors.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/abilene-emerson.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/abilene-emerson</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:55.923Z</t>
+  </si>
+  <si>
+    <t>Abilene Emerson | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories/abilene-emerson.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/dhaara-antani.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/dhaara-antani</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:50.332Z</t>
+  </si>
+  <si>
+    <t>Dhaara Antani | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories/dhaara-antani.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/harish-kilaru.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/harish-kilaru</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:57.858Z</t>
+  </si>
+  <si>
+    <t>Harish Kilaru | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories/harish-kilaru.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/jenna-malzahn.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/jenna-malzahn</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:59.941Z</t>
+  </si>
+  <si>
+    <t>Jenna Malzahn | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories/jenna-malzahn.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/kepriah-davis.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/student-stories/kepriah-davis</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:53.447Z</t>
+  </si>
+  <si>
+    <t>Kepriah Davis | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/student-stories/kepriah-davis.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/admissions.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/admissions</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:21.313Z</t>
+  </si>
+  <si>
+    <t>Admissions | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/admissions.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/curriculum.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/curriculum</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:17.106Z</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/curriculum.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/scholarships-financialaid-tuition.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/scholarships-financialaid-tuition</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:23.393Z</t>
+  </si>
+  <si>
+    <t>Scholarships, Financial Aid, and Tuition | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/scholarships-financialaid-tuition.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/student-life.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/student-life</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:19.185Z</t>
+  </si>
+  <si>
+    <t>Student Life | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/student-life.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/what-are-the-liberal-arts.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/what-are-the-liberal-arts</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:14.633Z</t>
+  </si>
+  <si>
+    <t>What Are the Liberal Arts? | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/what-are-the-liberal-arts-.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/academics.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/academics</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:16.787Z</t>
+  </si>
+  <si>
+    <t>Academics | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/academics.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admissions-and-requirements.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admissions-and-requirements</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:14.782Z</t>
+  </si>
+  <si>
+    <t>Admissions and Requirements | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/admissions-and-requirements.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admitted-students.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admitted-students</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:22.618Z</t>
+  </si>
+  <si>
+    <t>Admitted Students | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/admitted-students.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/student-life.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/student-life</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:19.854Z</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/student-life.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/admissions/undergraduate-application.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/undergraduate/admissions/undergraduate-application</t>
+  </si>
+  <si>
+    <t>2026-10-07T18:31:39.165Z</t>
+  </si>
+  <si>
+    <t>Undergraduate Application | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/admissions/undergraduate-application.html</t>
   </si>
 </sst>
 </file>
@@ -745,12 +1228,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
     <col min="10" max="11" width="50" customWidth="1"/>
@@ -1041,7 +1524,7 @@
         <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -1050,30 +1533,30 @@
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J9" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="K9" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
         <v>13</v>
@@ -1085,10 +1568,10 @@
         <v>13</v>
       </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
@@ -1097,7 +1580,7 @@
         <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J10" t="s">
         <v>13</v>
@@ -1108,10 +1591,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>13</v>
@@ -1123,30 +1606,30 @@
         <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="J11" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
         <v>13</v>
@@ -1155,7 +1638,7 @@
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
         <v>66</v>
@@ -1164,59 +1647,59 @@
         <v>15</v>
       </c>
       <c r="H12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" t="s">
         <v>67</v>
       </c>
-      <c r="I12" t="s">
-        <v>68</v>
-      </c>
       <c r="J12" t="s">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" t="s">
         <v>71</v>
       </c>
-      <c r="B13" t="s">
+      <c r="J13" t="s">
         <v>72</v>
       </c>
-      <c r="C13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="K13" t="s">
         <v>73</v>
-      </c>
-      <c r="G13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s">
-        <v>74</v>
-      </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
-      <c r="J13" t="s">
-        <v>76</v>
-      </c>
-      <c r="K13" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
         <v>13</v>
@@ -1228,62 +1711,62 @@
         <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G14" t="s">
         <v>15</v>
       </c>
       <c r="H14" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="I14" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="J14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="K14" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" t="s">
+        <v>81</v>
+      </c>
+      <c r="J15" t="s">
+        <v>82</v>
+      </c>
+      <c r="K15" t="s">
         <v>83</v>
-      </c>
-      <c r="B15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" t="s">
-        <v>13</v>
-      </c>
-      <c r="I15" t="s">
-        <v>87</v>
-      </c>
-      <c r="J15" t="s">
-        <v>13</v>
-      </c>
-      <c r="K15" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
@@ -1298,127 +1781,1282 @@
         <v>13</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G16" t="s">
         <v>15</v>
       </c>
       <c r="H16" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="I16" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="J16" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="K16" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
       </c>
       <c r="F17" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H17" t="s">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="I17" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="J17" t="s">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="K17" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>97</v>
+      </c>
+      <c r="I18" t="s">
+        <v>98</v>
+      </c>
+      <c r="J18" t="s">
+        <v>99</v>
+      </c>
+      <c r="K18" t="s">
         <v>100</v>
-      </c>
-      <c r="B18" t="s">
-        <v>101</v>
-      </c>
-      <c r="C18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s">
-        <v>102</v>
-      </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s">
-        <v>74</v>
-      </c>
-      <c r="I18" t="s">
-        <v>103</v>
-      </c>
-      <c r="J18" t="s">
-        <v>104</v>
-      </c>
-      <c r="K18" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>97</v>
+      </c>
+      <c r="I19" t="s">
+        <v>103</v>
+      </c>
+      <c r="J19" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>106</v>
       </c>
-      <c r="B19" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="B20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
         <v>107</v>
       </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" t="s">
+        <v>109</v>
+      </c>
+      <c r="J20" t="s">
+        <v>110</v>
+      </c>
+      <c r="K20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>108</v>
+      </c>
+      <c r="I21" t="s">
+        <v>114</v>
+      </c>
+      <c r="J21" t="s">
+        <v>115</v>
+      </c>
+      <c r="K21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" t="s">
+        <v>118</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
+        <v>108</v>
+      </c>
+      <c r="I22" t="s">
+        <v>119</v>
+      </c>
+      <c r="J22" t="s">
+        <v>120</v>
+      </c>
+      <c r="K22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>108</v>
+      </c>
+      <c r="I23" t="s">
+        <v>124</v>
+      </c>
+      <c r="J23" t="s">
+        <v>125</v>
+      </c>
+      <c r="K23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
+        <v>128</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>108</v>
+      </c>
+      <c r="I24" t="s">
+        <v>129</v>
+      </c>
+      <c r="J24" t="s">
+        <v>130</v>
+      </c>
+      <c r="K24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
+        <v>133</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
+        <v>134</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I25" t="s">
+        <v>135</v>
+      </c>
+      <c r="J25" t="s">
+        <v>136</v>
+      </c>
+      <c r="K25" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>108</v>
+      </c>
+      <c r="I26" t="s">
+        <v>140</v>
+      </c>
+      <c r="J26" t="s">
+        <v>141</v>
+      </c>
+      <c r="K26" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>143</v>
+      </c>
+      <c r="B27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
+        <v>144</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
         <v>16</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I27" t="s">
+        <v>145</v>
+      </c>
+      <c r="J27" t="s">
+        <v>146</v>
+      </c>
+      <c r="K27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" t="s">
+        <v>150</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
         <v>108</v>
       </c>
-      <c r="J19" t="s">
-        <v>109</v>
-      </c>
-      <c r="K19" t="s">
-        <v>110</v>
+      <c r="I28" t="s">
+        <v>151</v>
+      </c>
+      <c r="J28" t="s">
+        <v>152</v>
+      </c>
+      <c r="K28" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" t="s">
+        <v>149</v>
+      </c>
+      <c r="C29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
+        <v>155</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
+        <v>108</v>
+      </c>
+      <c r="I29" t="s">
+        <v>156</v>
+      </c>
+      <c r="J29" t="s">
+        <v>157</v>
+      </c>
+      <c r="K29" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B30" t="s">
+        <v>149</v>
+      </c>
+      <c r="C30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
+        <v>160</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>108</v>
+      </c>
+      <c r="I30" t="s">
+        <v>161</v>
+      </c>
+      <c r="J30" t="s">
+        <v>162</v>
+      </c>
+      <c r="K30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" t="s">
+        <v>165</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>108</v>
+      </c>
+      <c r="I31" t="s">
+        <v>166</v>
+      </c>
+      <c r="J31" t="s">
+        <v>167</v>
+      </c>
+      <c r="K31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
+        <v>170</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>108</v>
+      </c>
+      <c r="I32" t="s">
+        <v>171</v>
+      </c>
+      <c r="J32" t="s">
+        <v>172</v>
+      </c>
+      <c r="K32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
+        <v>175</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
+        <v>108</v>
+      </c>
+      <c r="I33" t="s">
+        <v>176</v>
+      </c>
+      <c r="J33" t="s">
+        <v>177</v>
+      </c>
+      <c r="K33" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
+        <v>180</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
+        <v>108</v>
+      </c>
+      <c r="I34" t="s">
+        <v>181</v>
+      </c>
+      <c r="J34" t="s">
+        <v>182</v>
+      </c>
+      <c r="K34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>184</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
+        <v>185</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>108</v>
+      </c>
+      <c r="I35" t="s">
+        <v>186</v>
+      </c>
+      <c r="J35" t="s">
+        <v>187</v>
+      </c>
+      <c r="K35" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s">
+        <v>190</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
+        <v>108</v>
+      </c>
+      <c r="I36" t="s">
+        <v>191</v>
+      </c>
+      <c r="J36" t="s">
+        <v>192</v>
+      </c>
+      <c r="K36" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>194</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" t="s">
+        <v>195</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>108</v>
+      </c>
+      <c r="I37" t="s">
+        <v>196</v>
+      </c>
+      <c r="J37" t="s">
+        <v>197</v>
+      </c>
+      <c r="K37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>199</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" t="s">
+        <v>200</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
+        <v>108</v>
+      </c>
+      <c r="I38" t="s">
+        <v>201</v>
+      </c>
+      <c r="J38" t="s">
+        <v>202</v>
+      </c>
+      <c r="K38" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>204</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" t="s">
+        <v>205</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
+        <v>108</v>
+      </c>
+      <c r="I39" t="s">
+        <v>206</v>
+      </c>
+      <c r="J39" t="s">
+        <v>207</v>
+      </c>
+      <c r="K39" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>209</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" t="s">
+        <v>210</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
+        <v>108</v>
+      </c>
+      <c r="I40" t="s">
+        <v>211</v>
+      </c>
+      <c r="J40" t="s">
+        <v>212</v>
+      </c>
+      <c r="K40" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>214</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
+        <v>215</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>108</v>
+      </c>
+      <c r="I41" t="s">
+        <v>216</v>
+      </c>
+      <c r="J41" t="s">
+        <v>217</v>
+      </c>
+      <c r="K41" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>219</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" t="s">
+        <v>220</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>108</v>
+      </c>
+      <c r="I42" t="s">
+        <v>221</v>
+      </c>
+      <c r="J42" t="s">
+        <v>222</v>
+      </c>
+      <c r="K42" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>224</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" t="s">
+        <v>225</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>108</v>
+      </c>
+      <c r="I43" t="s">
+        <v>226</v>
+      </c>
+      <c r="J43" t="s">
+        <v>227</v>
+      </c>
+      <c r="K43" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>229</v>
+      </c>
+      <c r="B44" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
+        <v>230</v>
+      </c>
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>108</v>
+      </c>
+      <c r="I44" t="s">
+        <v>231</v>
+      </c>
+      <c r="J44" t="s">
+        <v>177</v>
+      </c>
+      <c r="K44" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>233</v>
+      </c>
+      <c r="B45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C45" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" t="s">
+        <v>234</v>
+      </c>
+      <c r="G45" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" t="s">
+        <v>108</v>
+      </c>
+      <c r="I45" t="s">
+        <v>235</v>
+      </c>
+      <c r="J45" t="s">
+        <v>236</v>
+      </c>
+      <c r="K45" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>238</v>
+      </c>
+      <c r="B46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" t="s">
+        <v>13</v>
+      </c>
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" t="s">
+        <v>239</v>
+      </c>
+      <c r="G46" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" t="s">
+        <v>108</v>
+      </c>
+      <c r="I46" t="s">
+        <v>240</v>
+      </c>
+      <c r="J46" t="s">
+        <v>241</v>
+      </c>
+      <c r="K46" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>243</v>
+      </c>
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
+        <v>244</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>108</v>
+      </c>
+      <c r="I47" t="s">
+        <v>245</v>
+      </c>
+      <c r="J47" t="s">
+        <v>246</v>
+      </c>
+      <c r="K47" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>248</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
+        <v>249</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>108</v>
+      </c>
+      <c r="I48" t="s">
+        <v>250</v>
+      </c>
+      <c r="J48" t="s">
+        <v>251</v>
+      </c>
+      <c r="K48" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>253</v>
+      </c>
+      <c r="B49" t="s">
+        <v>149</v>
+      </c>
+      <c r="C49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
+        <v>254</v>
+      </c>
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
+        <v>108</v>
+      </c>
+      <c r="I49" t="s">
+        <v>255</v>
+      </c>
+      <c r="J49" t="s">
+        <v>256</v>
+      </c>
+      <c r="K49" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>258</v>
+      </c>
+      <c r="B50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
+        <v>259</v>
+      </c>
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
+        <v>108</v>
+      </c>
+      <c r="I50" t="s">
+        <v>260</v>
+      </c>
+      <c r="J50" t="s">
+        <v>261</v>
+      </c>
+      <c r="K50" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>263</v>
+      </c>
+      <c r="B51" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" t="s">
+        <v>264</v>
+      </c>
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>108</v>
+      </c>
+      <c r="I51" t="s">
+        <v>265</v>
+      </c>
+      <c r="J51" t="s">
+        <v>241</v>
+      </c>
+      <c r="K51" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>267</v>
+      </c>
+      <c r="B52" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
+        <v>268</v>
+      </c>
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" t="s">
+        <v>108</v>
+      </c>
+      <c r="I52" t="s">
+        <v>269</v>
+      </c>
+      <c r="J52" t="s">
+        <v>270</v>
+      </c>
+      <c r="K52" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>